<commit_message>
Update labels and add descriptions
</commit_message>
<xml_diff>
--- a/inst/extdata/ui_labels.xlsx
+++ b/inst/extdata/ui_labels.xlsx
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="97" uniqueCount="59">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="117" uniqueCount="69">
   <si>
     <t xml:space="preserve">This sheet contains UI labels to be translated into french. If the UI is update, new labels should be added here.</t>
   </si>
@@ -92,6 +92,9 @@
     <t xml:space="preserve">Create mitigation</t>
   </si>
   <si>
+    <t xml:space="preserve">Help</t>
+  </si>
+  <si>
     <t xml:space="preserve">Sector</t>
   </si>
   <si>
@@ -129,6 +132,33 @@
   </si>
   <si>
     <t xml:space="preserve">Messages</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Compiling report, this may take a minute...</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Message will disappear when your report is ready</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mitigation created</t>
+  </si>
+  <si>
+    <t xml:space="preserve">To activate a created mitigation, select in 'Mitigation Measures' sidebar.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">To create an additional mitigation, click on a new edge.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mitigations can affect multiple pathways.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">To create a multipathway mitigation use the same 'Name' but select a different pathway.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">To create a completely new mitigation, ensure that you use a different 'Name'.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">If more than one mitigation affects the same edge, only the most recently one will be shown on the diagram.</t>
   </si>
   <si>
     <t xml:space="preserve">Stressors/pressures associated with Activities/Components selected by user</t>
@@ -279,7 +309,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -293,6 +323,10 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -443,7 +477,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:B57"/>
+  <dimension ref="A1:B75"/>
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="35.61"/>
@@ -586,7 +620,7 @@
       </c>
     </row>
     <row r="20" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="1" t="s">
+      <c r="A20" s="4" t="s">
         <v>23</v>
       </c>
       <c r="B20" s="1" t="s">
@@ -594,251 +628,355 @@
       </c>
     </row>
     <row r="21" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="1" t="s">
+      <c r="B21" s="1"/>
+    </row>
+    <row r="22" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B22" s="1"/>
+    </row>
+    <row r="23" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A23" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="B21" s="1" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="22" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="1" t="s">
+      <c r="B23" s="1" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="24" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A24" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="B22" s="1" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="23" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B23" s="1"/>
-    </row>
-    <row r="24" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B24" s="1"/>
+      <c r="B24" s="1" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="25" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A25" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="B25" s="1" t="s">
+        <v>10</v>
+      </c>
     </row>
     <row r="26" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A26" s="1" t="s">
-        <v>26</v>
-      </c>
-      <c r="B26" s="1" t="s">
-        <v>27</v>
-      </c>
+      <c r="B26" s="1"/>
     </row>
     <row r="27" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A27" s="1" t="s">
-        <v>28</v>
-      </c>
-      <c r="B27" s="1" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="28" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A28" s="1" t="s">
-        <v>29</v>
-      </c>
-      <c r="B28" s="1" t="s">
-        <v>27</v>
-      </c>
+      <c r="B27" s="1"/>
     </row>
     <row r="29" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="1" t="s">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="B29" s="1" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="1" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="B30" s="1" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="1" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="B31" s="1" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="1" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="B32" s="1" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B33" s="1"/>
+      <c r="A33" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="B33" s="1" t="s">
+        <v>28</v>
+      </c>
     </row>
     <row r="34" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="B34" s="1" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="35" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A35" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="B34" s="1" t="s">
-        <v>35</v>
+      <c r="B35" s="1" t="s">
+        <v>28</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A36" s="1" t="s">
-        <v>36</v>
-      </c>
-      <c r="B36" s="1" t="s">
-        <v>37</v>
-      </c>
+      <c r="B36" s="1"/>
     </row>
     <row r="37" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="1" t="s">
-        <v>38</v>
+        <v>35</v>
       </c>
       <c r="B37" s="1" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="38" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A38" s="1" t="s">
         <v>37</v>
+      </c>
+      <c r="B38" s="1" t="s">
+        <v>36</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="1" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B39" s="1" t="s">
-        <v>40</v>
+        <v>36</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="1" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="B40" s="1" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="41" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A41" s="1" t="s">
         <v>40</v>
+      </c>
+      <c r="B41" s="1" t="s">
+        <v>36</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="1" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="B42" s="1" t="s">
-        <v>17</v>
+        <v>36</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A43" s="1" t="s">
-        <v>43</v>
-      </c>
-      <c r="B43" s="1" t="s">
-        <v>17</v>
-      </c>
+      <c r="B43" s="1"/>
     </row>
     <row r="44" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="1" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="B44" s="1" t="s">
-        <v>17</v>
+        <v>23</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A45" s="1" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="B45" s="1" t="s">
-        <v>17</v>
+        <v>23</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A46" s="1" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="B46" s="1" t="s">
-        <v>17</v>
+        <v>23</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A47" s="1" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="B47" s="1" t="s">
-        <v>17</v>
+        <v>23</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A48" s="1" t="s">
-        <v>48</v>
-      </c>
-      <c r="B48" s="1" t="s">
-        <v>49</v>
-      </c>
+      <c r="B48" s="1"/>
     </row>
     <row r="49" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A49" s="1" t="s">
-        <v>50</v>
-      </c>
-      <c r="B49" s="1" t="s">
-        <v>49</v>
-      </c>
+      <c r="B49" s="1"/>
     </row>
     <row r="50" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A50" s="1" t="s">
-        <v>51</v>
-      </c>
-      <c r="B50" s="1" t="s">
-        <v>49</v>
-      </c>
+      <c r="B50" s="1"/>
     </row>
     <row r="51" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A51" s="1" t="s">
-        <v>52</v>
-      </c>
-      <c r="B51" s="1" t="s">
-        <v>17</v>
-      </c>
+      <c r="B51" s="1"/>
     </row>
     <row r="52" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A52" s="1" t="s">
-        <v>53</v>
-      </c>
-      <c r="B52" s="1" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="53" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A53" s="1" t="s">
-        <v>54</v>
-      </c>
-      <c r="B53" s="1" t="s">
-        <v>17</v>
-      </c>
+      <c r="B52" s="1"/>
     </row>
     <row r="54" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A54" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="B54" s="1" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="55" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A55" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="B55" s="1" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="57" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A57" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="B57" s="1" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="58" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A58" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="B58" s="1" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="60" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A60" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="B60" s="1" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="61" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A61" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="B61" s="1" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="62" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A62" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="B62" s="1" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="63" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A63" s="1" t="s">
         <v>55</v>
       </c>
-      <c r="B54" s="1" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="55" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A55" s="3" t="s">
+      <c r="B63" s="1" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="64" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A64" s="1" t="s">
         <v>56</v>
       </c>
-      <c r="B55" s="1" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="56" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A56" s="3" t="s">
+      <c r="B64" s="1" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="65" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A65" s="1" t="s">
         <v>57</v>
       </c>
-      <c r="B56" s="1" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="57" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A57" s="3" t="s">
+      <c r="B65" s="1" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="66" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A66" s="1" t="s">
         <v>58</v>
       </c>
-      <c r="B57" s="1" t="s">
+      <c r="B66" s="1" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="67" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A67" s="1" t="s">
+        <v>60</v>
+      </c>
+      <c r="B67" s="1" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="68" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A68" s="1" t="s">
+        <v>61</v>
+      </c>
+      <c r="B68" s="1" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="69" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A69" s="1" t="s">
+        <v>62</v>
+      </c>
+      <c r="B69" s="1" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="70" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A70" s="1" t="s">
+        <v>63</v>
+      </c>
+      <c r="B70" s="1" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="71" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A71" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="B71" s="1" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="72" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A72" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="B72" s="1" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="73" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A73" s="3" t="s">
+        <v>66</v>
+      </c>
+      <c r="B73" s="1" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="74" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A74" s="3" t="s">
+        <v>67</v>
+      </c>
+      <c r="B74" s="1" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="75" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A75" s="3" t="s">
+        <v>68</v>
+      </c>
+      <c r="B75" s="1" t="s">
         <v>17</v>
       </c>
     </row>

</xml_diff>